<commit_message>
Remove port fields from Excel template - ports loaded from .env files
- Removed Source Port and Target Port from Excel template fields
- Made source_port and target_port Optional in ValidationConfig
- Parser now treats ports as optional (loaded from .env if not in Excel)
- Updated create_excel_template.py to reflect .env-only design
- Regenerated validation_template.xlsx without port fields

Ports are now ONLY in .env files, not in Excel.
This aligns with the host-specific credential management design.

Co-Authored-By: Claude Sonnet 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/validation_template.xlsx
+++ b/examples/validation_template.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -547,522 +547,478 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Source Port</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>3085</v>
-      </c>
-      <c r="C5" t="n">
-        <v>1521</v>
-      </c>
-      <c r="D5" t="n">
-        <v>5480</v>
-      </c>
-      <c r="E5" t="n">
-        <v>3085</v>
-      </c>
-      <c r="F5" t="n">
-        <v>3085</v>
+          <t>Source Database Name</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>OrderDB</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>SALES_DB</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>cidpr</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>OrderDB</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>SalesDB</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Source Database Name</t>
+          <t>Source Schema Name</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>OrderDB</t>
+          <t>dbo</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>SALES_DB</t>
+          <t>SALES</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>cidpr</t>
+          <t>stgprd</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>OrderDB</t>
+          <t>dbo</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>SalesDB</t>
+          <t>dbo</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Source Schema Name</t>
+          <t>Source Table Name</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>dbo</t>
+          <t>Orders</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>SALES</t>
+          <t>TRANSACTIONS</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>stgprd</t>
+          <t>PRODUCT_MASTER</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>dbo</t>
+          <t>Orders</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>dbo</t>
+          <t>Sales</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Source Table Name</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Orders</t>
-        </is>
-      </c>
+          <t>Source Column Name</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
-          <t>TRANSACTIONS</t>
+          <t>AMOUNT</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>PRODUCT_MASTER</t>
+          <t>PRODUCT_ID</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Orders</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Sales</t>
-        </is>
-      </c>
+          <t>ORDER_TOTAL</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Source Column Name</t>
+          <t>Source Column Expression</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>AMOUNT</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>PRODUCT_ID</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>ORDER_TOTAL</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Price * Quantity</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Source Column Expression</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
+          <t>Source Filter</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>order_date &gt;= '2024-01-01'</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>TRANSACTION_DATE &gt;= TO_DATE('2024-01-01', 'YYYY-MM-DD')</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>IS_ACTIVE = TRUE</t>
+        </is>
+      </c>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Price * Quantity</t>
+          <t>REGION = 'WEST'</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Source Filter</t>
+          <t>Target Type</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>order_date &gt;= '2024-01-01'</t>
+          <t>Snowflake</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>TRANSACTION_DATE &gt;= TO_DATE('2024-01-01', 'YYYY-MM-DD')</t>
+          <t>Snowflake</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>IS_ACTIVE = TRUE</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr"/>
+          <t>SQLServer</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Netezza</t>
+        </is>
+      </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>REGION = 'WEST'</t>
+          <t>Netezza</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Target Type</t>
+          <t>Target Host Name</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Snowflake</t>
+          <t>snowflake-prod</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Snowflake</t>
+          <t>snowflake-prod</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>SQLServer</t>
+          <t>p8054</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Netezza</t>
+          <t>nz-db-ut</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Netezza</t>
+          <t>nz-db-ut</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Target Host Name</t>
+          <t>Target Database Name</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>snowflake-prod</t>
+          <t>ANALYTICS</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>snowflake-prod</t>
+          <t>ANALYTICS</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>p8054</t>
+          <t>BDM Archive</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>nz-db-ut</t>
+          <t>cidpr</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>nz-db-ut</t>
+          <t>cidpr</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Target Port</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>443</v>
-      </c>
-      <c r="C14" t="n">
-        <v>443</v>
-      </c>
-      <c r="D14" t="n">
-        <v>3085</v>
-      </c>
-      <c r="E14" t="n">
-        <v>5480</v>
-      </c>
-      <c r="F14" t="n">
-        <v>5480</v>
+          <t>Target Schema Name</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>PUBLIC</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>SALES</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>dbo</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>stgprd</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>stgprd</t>
+        </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Target Database Name</t>
+          <t>Target Table Name</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ANALYTICS</t>
+          <t>ORDERS_FACT</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ANALYTICS</t>
+          <t>TRANSACTIONS</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>BDM Archive</t>
+          <t>PRODUCT_DIM</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>cidpr</t>
+          <t>ORDERS</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>cidpr</t>
+          <t>Sales_Fact</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Target Schema Name</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>PUBLIC</t>
-        </is>
-      </c>
+          <t>Target Column Name</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr">
         <is>
-          <t>SALES</t>
+          <t>AMOUNT</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>dbo</t>
+          <t>PRODUCT_ID</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>stgprd</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>stgprd</t>
-        </is>
-      </c>
+          <t>ORDER_TOTAL</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Target Table Name</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>ORDERS_FACT</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>TRANSACTIONS</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>PRODUCT_DIM</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>ORDERS</t>
-        </is>
-      </c>
+          <t>Target Column Expression</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Sales_Fact</t>
+          <t>Price * Quantity</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Target Column Name</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr"/>
+          <t>Target Filter</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ORDER_DATE &gt;= '2024-01-01'</t>
+        </is>
+      </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>AMOUNT</t>
+          <t>TRANSACTION_DATE &gt;= '2024-01-01'</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>PRODUCT_ID</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>ORDER_TOTAL</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr"/>
+          <t>IS_ACTIVE = 1</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>REGION = 'WEST'</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Target Column Expression</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
+          <t>Rule Type</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>COUNT_STAR</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>SUM</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>COUNT_DISTINCT</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>AVG</t>
+        </is>
+      </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Price * Quantity</t>
+          <t>SUM</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Target Filter</t>
+          <t>Threshold Type</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ORDER_DATE &gt;= '2024-01-01'</t>
+          <t>EXACT</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>TRANSACTION_DATE &gt;= '2024-01-01'</t>
+          <t>PERCENTAGE</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>IS_ACTIVE = 1</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr"/>
+          <t>EXACT</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>ABSOLUTE</t>
+        </is>
+      </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>REGION = 'WEST'</t>
+          <t>PERCENTAGE</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Rule Type</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>COUNT_STAR</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>SUM</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>COUNT_DISTINCT</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>AVG</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>SUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Threshold Type</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>EXACT</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>PERCENTAGE</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>EXACT</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>ABSOLUTE</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>PERCENTAGE</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
           <t>Threshold Value</t>
         </is>
       </c>
-      <c r="B23" t="n">
+      <c r="B21" t="n">
         <v>0</v>
       </c>
-      <c r="C23" t="n">
+      <c r="C21" t="n">
         <v>0.01</v>
       </c>
-      <c r="D23" t="n">
+      <c r="D21" t="n">
         <v>0</v>
       </c>
-      <c r="E23" t="n">
+      <c r="E21" t="n">
         <v>5</v>
       </c>
-      <c r="F23" t="n">
+      <c r="F21" t="n">
         <v>0.02</v>
       </c>
     </row>

</xml_diff>